<commit_message>
feat: add roof correlation marks in quality house workbook
Co-authored-by: Hi-ppie <107366561+Hi-ppie@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/дом качества — экономичная термокружка для студентов.xlsx
+++ b/дом качества — экономичная термокружка для студентов.xlsx
@@ -1135,6 +1135,11 @@
       <c r="E5" s="27" t="n"/>
       <c r="F5" s="35" t="n"/>
       <c r="G5" s="69" t="n"/>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="J5" s="70" t="inlineStr">
         <is>
           <t>Положительно</t>
@@ -1165,7 +1170,16 @@
       <c r="D6" s="69" t="n"/>
       <c r="E6" s="27" t="n"/>
       <c r="F6" s="35" t="n"/>
-      <c r="G6" s="69" t="n"/>
+      <c r="G6" s="69" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
       <c r="K6" s="31" t="n"/>
       <c r="L6" s="32" t="n"/>
     </row>
@@ -1174,8 +1188,21 @@
       <c r="C7" s="4" t="n"/>
       <c r="D7" s="69" t="n"/>
       <c r="E7" s="27" t="n"/>
-      <c r="F7" s="35" t="n"/>
-      <c r="G7" s="69" t="n"/>
+      <c r="F7" s="35" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G7" s="69" t="inlineStr">
+        <is>
+          <t>.</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
       <c r="J7" s="71" t="inlineStr">
         <is>
           <t>Соотношение:</t>
@@ -1188,10 +1215,26 @@
       <c r="B8" s="69" t="n"/>
       <c r="C8" s="27" t="n"/>
       <c r="D8" s="69" t="n"/>
-      <c r="E8" s="27" t="n"/>
-      <c r="F8" s="35" t="n"/>
-      <c r="G8" s="69" t="n"/>
-      <c r="H8" s="27" t="n"/>
+      <c r="E8" s="27" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F8" s="35" t="inlineStr">
+        <is>
+          <t>+</t>
+        </is>
+      </c>
+      <c r="G8" s="69" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H8" s="27" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="J8" s="33" t="n">
         <v>9</v>
       </c>
@@ -1931,7 +1974,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Приоритеты улучшения: удержание тепла, герметичность/эргономика крышки и снижение цены при сохранении прочности и экологичности.</t>
+          <t>Приоритеты улучшения: максимизировать сохранение тепла и надежность герметичной крышки, затем снижать цену без потери прочности и экологичности материалов.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: replace roof dot markers with explicit correlation signs
Co-authored-by: Hi-ppie <107366561+Hi-ppie@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/дом качества — экономичная термокружка для студентов.xlsx
+++ b/дом качества — экономичная термокружка для студентов.xlsx
@@ -996,7 +996,7 @@
                 <a:latin typeface="+mn-lt"/>
                 <a:cs typeface="Arial"/>
               </a:rPr>
-              <a:t>.</a:t>
+              <a:t>+</a:t>
             </a:r>
           </a:p>
         </xdr:txBody>
@@ -1049,7 +1049,7 @@
                 <a:latin typeface="+mn-lt"/>
                 <a:cs typeface="Arial"/>
               </a:rPr>
-              <a:t>.</a:t>
+              <a:t>-</a:t>
             </a:r>
           </a:p>
         </xdr:txBody>
@@ -1102,7 +1102,7 @@
                 <a:latin typeface="+mn-lt"/>
                 <a:cs typeface="Arial"/>
               </a:rPr>
-              <a:t>.</a:t>
+              <a:t>+</a:t>
             </a:r>
           </a:p>
         </xdr:txBody>
@@ -1155,7 +1155,7 @@
                 <a:latin typeface="+mn-lt"/>
                 <a:cs typeface="Arial"/>
               </a:rPr>
-              <a:t>.</a:t>
+              <a:t>-</a:t>
             </a:r>
           </a:p>
         </xdr:txBody>
@@ -1208,7 +1208,7 @@
                 <a:latin typeface="+mn-lt"/>
                 <a:cs typeface="Arial"/>
               </a:rPr>
-              <a:t>.</a:t>
+              <a:t>+</a:t>
             </a:r>
           </a:p>
         </xdr:txBody>
@@ -1261,7 +1261,7 @@
                 <a:latin typeface="+mn-lt"/>
                 <a:cs typeface="Arial"/>
               </a:rPr>
-              <a:t>.</a:t>
+              <a:t>-</a:t>
             </a:r>
           </a:p>
         </xdr:txBody>
@@ -1314,7 +1314,7 @@
                 <a:latin typeface="+mn-lt"/>
                 <a:cs typeface="Arial"/>
               </a:rPr>
-              <a:t>.</a:t>
+              <a:t>+</a:t>
             </a:r>
           </a:p>
         </xdr:txBody>
@@ -1367,7 +1367,7 @@
                 <a:latin typeface="+mn-lt"/>
                 <a:cs typeface="Arial"/>
               </a:rPr>
-              <a:t>.</a:t>
+              <a:t>-</a:t>
             </a:r>
           </a:p>
         </xdr:txBody>
@@ -1420,7 +1420,7 @@
                 <a:latin typeface="+mn-lt"/>
                 <a:cs typeface="Arial"/>
               </a:rPr>
-              <a:t>.</a:t>
+              <a:t>+</a:t>
             </a:r>
           </a:p>
         </xdr:txBody>
@@ -1473,7 +1473,7 @@
                 <a:latin typeface="+mn-lt"/>
                 <a:cs typeface="Arial"/>
               </a:rPr>
-              <a:t>.</a:t>
+              <a:t>-</a:t>
             </a:r>
           </a:p>
         </xdr:txBody>

</xml_diff>